<commit_message>
Add ERP phase 2 master data
</commit_message>
<xml_diff>
--- a/svet akcija/outputs/Svet_akcija_product_inventory_and_UX_plan.xlsx
+++ b/svet akcija/outputs/Svet_akcija_product_inventory_and_UX_plan.xlsx
@@ -20022,7 +20022,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Set za čišćenje PowerMop^J ljubičasta.docx</t>
+          <t>Set za čišćenje PowerMop^J ljubičasta.docx</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
@@ -20046,7 +20046,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Set za čišćenje PowerMop^J ljubičasta.docx</t>
+          <t>Set za čišćenje PowerMop^J ljubičasta.docx</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
@@ -20070,7 +20070,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Set za čišćenje Flexi Mop Pro.docx</t>
+          <t>Set za čišćenje Flexi Mop Pro.docx</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
@@ -20094,7 +20094,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Set za čišćenje UltraMop Duo, plava.docx</t>
+          <t>Set za čišćenje UltraMop Duo, plava.docx</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
@@ -20262,7 +20262,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Set za čišćenje Smart Spin.docx</t>
+          <t>Set za čišćenje Smart Spin.docx</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
@@ -20310,7 +20310,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Praško Dust Master.docx</t>
+          <t>Praško Dust Master.docx</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
@@ -20334,7 +20334,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Komplet za čišćenje Dust Away 360º.docx</t>
+          <t>Komplet za čišćenje Dust Away 360º.docx</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
@@ -20358,7 +20358,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Brisač stakla Pure Stream Pro.docx</t>
+          <t>Brisač stakla Pure Stream Pro.docx</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
@@ -20406,7 +20406,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Četkasti čistač za čaše sa dvostrukim glavama Glass Mate X.docx</t>
+          <t>Četkasti čistač za čaše sa dvostrukim glavama Glass Mate X.docx</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
@@ -20430,7 +20430,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Super secko Fresh Cut za povrće sa praktičnim posudama sa 15 nastavaka.docx</t>
+          <t>Super secko Fresh Cut za povrće sa praktičnim posudama sa 15 nastavaka.docx</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
@@ -20554,7 +20554,7 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>1019</v>
+        <v>129</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>4</v>
@@ -20578,7 +20578,7 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>984</v>
+        <v>129</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>5</v>
@@ -20602,7 +20602,7 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>1347</v>
+        <v>129</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>5</v>
@@ -20626,7 +20626,7 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>1137</v>
+        <v>129</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>6</v>
@@ -20650,7 +20650,7 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>1135</v>
+        <v>129</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>6</v>
@@ -20674,7 +20674,7 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>1019</v>
+        <v>129</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>4</v>
@@ -20698,7 +20698,7 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>1007</v>
+        <v>129</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>3</v>
@@ -20722,7 +20722,7 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>1085</v>
+        <v>129</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>7</v>
@@ -20746,7 +20746,7 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>1070</v>
+        <v>129</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>6</v>
@@ -20770,7 +20770,7 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>1003</v>
+        <v>129</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>6</v>
@@ -20794,7 +20794,7 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>2252</v>
+        <v>129</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>6</v>
@@ -20818,7 +20818,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1935</v>
+        <v>129</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>10</v>
@@ -20842,7 +20842,7 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>1956</v>
+        <v>129</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>10</v>
@@ -20866,7 +20866,7 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>906</v>
+        <v>129</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>5</v>
@@ -20890,7 +20890,7 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>1194</v>
+        <v>129</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>7</v>
@@ -20914,7 +20914,7 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>2267</v>
+        <v>129</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>7</v>
@@ -20938,7 +20938,7 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>1577</v>
+        <v>129</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>7</v>
@@ -20958,11 +20958,11 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Bežični usisivač Elegance, 120W, 600ml.docx</t>
+          <t>Bežični usisivač Elegance, 120W, 600ml.docx</t>
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>1544</v>
+        <v>129</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>7</v>
@@ -20986,7 +20986,7 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>1484</v>
+        <v>129</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>9</v>
@@ -21010,7 +21010,7 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>1750</v>
+        <v>129</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>5</v>
@@ -21034,7 +21034,7 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>1365</v>
+        <v>129</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>4</v>
@@ -21058,7 +21058,7 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>1355</v>
+        <v>129</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>5</v>
@@ -21082,7 +21082,7 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>1379</v>
+        <v>129</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>5</v>
@@ -21106,7 +21106,7 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>717</v>
+        <v>129</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>1</v>
@@ -21130,7 +21130,7 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>717</v>
+        <v>129</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>1</v>
@@ -21154,7 +21154,7 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>812</v>
+        <v>129</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>1</v>
@@ -21178,7 +21178,7 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>812</v>
+        <v>129</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>1</v>
@@ -21202,7 +21202,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>670</v>
+        <v>129</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>1</v>
@@ -21226,7 +21226,7 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>670</v>
+        <v>129</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>1</v>
@@ -21250,7 +21250,7 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>670</v>
+        <v>129</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>1</v>
@@ -21274,7 +21274,7 @@
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>670</v>
+        <v>129</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>1</v>
@@ -21298,7 +21298,7 @@
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>657</v>
+        <v>129</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>1</v>
@@ -21322,7 +21322,7 @@
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>657</v>
+        <v>129</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>1</v>
@@ -21346,7 +21346,7 @@
         </is>
       </c>
       <c r="D81" s="2" t="n">
-        <v>657</v>
+        <v>129</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>1</v>
@@ -21370,7 +21370,7 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>1144</v>
+        <v>129</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>10</v>
@@ -21394,7 +21394,7 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>1713</v>
+        <v>129</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>27</v>
@@ -21418,7 +21418,7 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>1064</v>
+        <v>129</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>12</v>
@@ -21442,7 +21442,7 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>1176</v>
+        <v>129</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>16</v>
@@ -21466,7 +21466,7 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>1190</v>
+        <v>129</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>10</v>
@@ -21490,7 +21490,7 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>1285</v>
+        <v>129</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>10</v>
@@ -21514,7 +21514,7 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>970</v>
+        <v>129</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>15</v>
@@ -21538,7 +21538,7 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>1289</v>
+        <v>129</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>6</v>
@@ -21562,7 +21562,7 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>1670</v>
+        <v>129</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>9</v>
@@ -21586,7 +21586,7 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>1782</v>
+        <v>129</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>10</v>
@@ -21610,7 +21610,7 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>1668</v>
+        <v>129</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>10</v>
@@ -21634,7 +21634,7 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>1780</v>
+        <v>129</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>12</v>
@@ -21658,7 +21658,7 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>1143</v>
+        <v>129</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>23</v>
@@ -21682,7 +21682,7 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>1143</v>
+        <v>129</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>23</v>
@@ -21706,7 +21706,7 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>1232</v>
+        <v>129</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>10</v>
@@ -21730,7 +21730,7 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>1015</v>
+        <v>129</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>7</v>
@@ -21754,7 +21754,7 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>1143</v>
+        <v>129</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>10</v>
@@ -21778,7 +21778,7 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>1305</v>
+        <v>129</v>
       </c>
       <c r="E99" s="2" t="n">
         <v>7</v>
@@ -21802,7 +21802,7 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>984</v>
+        <v>129</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>5</v>
@@ -21826,7 +21826,7 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>908</v>
+        <v>129</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>6</v>
@@ -21850,7 +21850,7 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>1062</v>
+        <v>129</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>10</v>
@@ -21874,7 +21874,7 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>1215</v>
+        <v>129</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>2</v>
@@ -21898,7 +21898,7 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>1062</v>
+        <v>129</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>5</v>
@@ -21922,7 +21922,7 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>1031</v>
+        <v>129</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>3</v>
@@ -21946,7 +21946,7 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>1056</v>
+        <v>129</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>2</v>
@@ -21970,7 +21970,7 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>1159</v>
+        <v>129</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>3</v>
@@ -21994,7 +21994,7 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>1163</v>
+        <v>129</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>3</v>
@@ -22018,7 +22018,7 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>815</v>
+        <v>129</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>6</v>
@@ -22042,7 +22042,7 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>817</v>
+        <v>129</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>5</v>
@@ -22066,7 +22066,7 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>1015</v>
+        <v>129</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>6</v>
@@ -22090,7 +22090,7 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>1330</v>
+        <v>129</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>7</v>
@@ -22114,7 +22114,7 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>1076</v>
+        <v>129</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>6</v>
@@ -22138,7 +22138,7 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>1090</v>
+        <v>129</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>7</v>
@@ -22162,7 +22162,7 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>1365</v>
+        <v>129</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>19</v>
@@ -22186,7 +22186,7 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>1196</v>
+        <v>129</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>7</v>

</xml_diff>

<commit_message>
Finish Svet Akcija phase 2 import safeguards
</commit_message>
<xml_diff>
--- a/svet akcija/outputs/Svet_akcija_product_inventory_and_UX_plan.xlsx
+++ b/svet akcija/outputs/Svet_akcija_product_inventory_and_UX_plan.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Products_exact'!$A$1:$Q$210</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Categories'!$A$1:$C$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Groups'!$A$1:$D$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Data_checks'!$A$1:$F$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Data_checks'!$A$1:$F$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Duplicate_checks'!$A$1:$G$125</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'UX_plan'!$A$1:$E$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Implementation_mapping'!$A$1:$E$18</definedName>
@@ -13509,7 +13509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -13999,59 +13999,67 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Empty stock/logistics fields</t>
+          <t>Git LFS pointer long descriptions</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>206</v>
+        <v>69</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>210019, 210003, 210022, 1040, 1025, 1114, 1116, 210000, 210001, 1033, 210009, 1034, 1095, 1035, 210013, 210011, 210012, 210010, 1112, 210020, 210024, 1075, 1044, 1074, 1076, 210006, 210023, 1045, 1106, 210014, 1049, 1053, 1111, 210025, 210016, 210015, 210017, 210018, 210021, 1037, 1036, 1097, 1096, 1109, 210002, 1080, 1078, 1077, 1039, 1079, 1027, 1181, 1110, 210004, 210005, 1098, 1041, 1099, 1100, 1101, 1042, 1107, 1022, 1031, 1032, 1029, 1030, 1043, 210007, 1023, 1024, 1038, 1050, 1115, 1048, 1047, 1028, 1182, 1183, 1046 ... (+126 more)</t>
+          <t>1114, 1116, 1112, 1106, 1111, 1109, 1110, 1107, 1115, 1108, 1141, 1139, 1142, 1140, 1122, 1123, 1120, 1121, 1124, 1125, 1126, 1127, 1128, 1129, 1130, 1136, 1131, 1133, 1134, 1135, 1132, 1137, 1162, 1083, 1089, 1161, 1085, 1164, 1165, 1144, 1143, 1160, 1138, 1118, 1119, 1117, 1088, 1086, 1084, 1163, 1149, 1146, 1103, 1145, 1148, 1102, 1170, 1171, 1169, 1172, 1104, 1168, 1166, 1167, 1147, 1105, 1151, 1173, 1150</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 80, 81 ... (+126 more)</t>
+          <t>7, 8, 20, 30, 34, 45, 54, 63, 75, 86, 93, 100, 104, 107, 108, 109, 110, 111, 112, 113, 114, 115, 116, 117, 118, 120, 121, 122, 123, 124, 125, 126, 127, 133, 134, 138, 142, 143, 144, 145, 146, 148, 153, 155, 156, 157, 161, 162, 164, 169, 170, 171, 172, 173, 174, 175, 176, 177, 180, 183, 184, 196, 197, 198, 200, 201, 202, 208, 210</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Rows where 'DC (lager)' is empty/null.</t>
+          <t>Product DOCX files that extracted as Git LFS pointer metadata instead of real description text.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Do not expose DC (lager) publicly; ask client if a separate public availability field will be provided.</t>
+          <t>Fetch the real LFS-backed DOCX files or replace them before publishing long product copy.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Action price higher than regular price</t>
+          <t>Empty stock/logistics fields</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr"/>
+        <v>206</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>210019, 210003, 210022, 1040, 1025, 1114, 1116, 210000, 210001, 1033, 210009, 1034, 1095, 1035, 210013, 210011, 210012, 210010, 1112, 210020, 210024, 1075, 1044, 1074, 1076, 210006, 210023, 1045, 1106, 210014, 1049, 1053, 1111, 210025, 210016, 210015, 210017, 210018, 210021, 1037, 1036, 1097, 1096, 1109, 210002, 1080, 1078, 1077, 1039, 1079, 1027, 1181, 1110, 210004, 210005, 1098, 1041, 1099, 1100, 1101, 1042, 1107, 1022, 1031, 1032, 1029, 1030, 1043, 210007, 1023, 1024, 1038, 1050, 1115, 1048, 1047, 1028, 1182, 1183, 1046 ... (+126 more)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 80, 81 ... (+126 more)</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Rows where numeric Akcijska MPC is greater than numeric MPC redovna.</t>
+          <t>Rows where 'DC (lager)' is empty/null.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Ask client to confirm price data before publishing these SKUs.</t>
+          <t>Missing stock imports as unavailable; ask the client to provide launch-approved SKU-level availability before publishing.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Identical regular and action price</t>
+          <t>Action price higher than regular price</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -14061,19 +14069,19 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Rows where numeric Akcijska MPC equals numeric MPC redovna.</t>
+          <t>Rows where numeric Akcijska MPC is greater than numeric MPC redovna.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Ask client whether these are truly action items or should display as regular-price products.</t>
+          <t>Ask client to confirm price data before publishing these SKUs.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Suspicious placeholder values</t>
+          <t>Identical regular and action price</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
@@ -14083,129 +14091,225 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Detected values exactly matching placeholder tokens: 9, 0, /, -, N/A, NA.</t>
+          <t>Rows where numeric Akcijska MPC equals numeric MPC redovna.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Do not display these values publicly unless the client confirms the value is meaningful.</t>
+          <t>Ask client whether these are truly action items or should display as regular-price products.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Numeric action-date values</t>
+          <t>Expired campaign price window</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
+        <v>209</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>210019, 210003, 210022, 1040, 1025, 1114, 1116, 210000, 210001, 1033, 210009, 1034, 1095, 1035, 210013, 210011, 210012, 210010, 1112, 210020, 210024, 1075, 1044, 1074, 1076, 210006, 210023, 1045, 1106, 210014, 1049, 1053, 1111, 210025, 210016, 210015, 210017, 210018, 210021, 1037, 1036, 1097, 1096, 1109, 210002, 1080, 1078, 1077, 1039, 1079, 1027, 1181, 1110, 210004, 210005, 1098, 1041, 1099, 1100, 1101, 1042, 1107, 1022, 1031, 1032, 1029, 1030, 1043, 210007, 1023, 1024, 1038, 1050, 1115, 1048, 1047, 1028, 1182, 1183, 1046 ... (+129 more)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 80, 81 ... (+129 more)</t>
+        </is>
+      </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Rows where action validity date fields are plain numbers in the exported workbook.</t>
+          <t>Rows with a discounted Akcijska MPC whose validity end date is before the report generation date.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>If present, ask whether Excel serial dates should be converted for display; keep source values unchanged.</t>
+          <t>Do not import these as sale prices; request current owner-approved campaign dates or publish regular price only.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Repeated non-descriptive review: Kolekcija (brend)</t>
+          <t>Invalid campaign date window</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>110</v>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>210019, 210003, 210022, 1040, 210000, 210001, 1033, 210009, 1034, 1095, 1035, 210013, 210011, 210012, 210010, 1112, 210020, 210024, 1075, 1044, 1074, 1076, 210006, 210023, 1045, 1106, 210014, 1049, 1053, 210025, 210016, 210015, 210017, 210018, 210021, 1037, 1036, 1097, 1096, 1109, 210002, 1080, 1078, 1077, 1039, 1079, 1110, 210004, 210005, 1098, 1041, 1099, 1100, 1101, 1042, 1043, 210007, 1038, 1050, 1115, 1048, 1047, 1046, 210008, 1011, 1014, 1010, 1013, 1009, 1141, 1012, 1005, 1008, 1004, 1007, 1003, 1139, 1006, 1017, 1018 ... (+30 more)</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>2, 3, 4, 5, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 33, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 54, 55, 56, 57, 58, 59, 60, 61, 62, 69, 70, 73, 74, 75, 76, 77, 81, 82, 88, 89, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99, 100, 101, 102, 103 ... (+30 more)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Frequently repeated values found: EVONEK (26), RAF (28), BEAUTECH (10), ORBITA (20), POMPEA MIMI (11), SPARKLE (15)</t>
+          <t>Rows with discounted Akcijska MPC but missing or unparsable campaign validity dates.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Confirm these are valid customer-facing filter/spec values before exposing as filters.</t>
+          <t>Fix campaign dates before importing a sale price.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Repeated non-descriptive review: Boja 1</t>
+          <t>Future campaign price window</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>112</v>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>210019, 210003, 1025, 1114, 210000, 210001, 1034, 210011, 210012, 1112, 210020, 210024, 1076, 210006, 210023, 1045, 210014, 1049, 1053, 1111, 210025, 210016, 210017, 210018, 1037, 1036, 1109, 210002, 1080, 1078, 1027, 1110, 210004, 210005, 1041, 1042, 1107, 1022, 1032, 1030, 1043, 210007, 1023, 1024, 1038, 1050, 1028, 1046, 210008, 1020, 1019, 1021, 1108, 1026, 1011, 1014, 1010, 1013, 1009, 1141, 1012, 1005, 1008, 1004, 1007, 1003, 1139, 1006, 1017, 1018, 1142, 1015, 1016, 1140, 1135, 1132, 210031, 1156, 1153, 1089 ... (+32 more)</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>2, 3, 6, 7, 9, 10, 13, 17, 18, 20, 21, 22, 26, 27, 28, 29, 31, 32, 33, 34, 35, 36, 38, 39, 41, 42, 45, 46, 47, 48, 52, 54, 55, 56, 58, 62, 63, 64, 66, 68, 69, 70, 71, 72, 73, 74, 78, 81, 82, 83, 84, 85, 86, 87, 88, 89, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99, 100, 101, 102, 103, 104, 105, 106, 107, 124, 125, 129, 131, 132, 134 ... (+32 more)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Frequently repeated values found: crna (37), bela (29), siva (29), plava (17)</t>
+          <t>Rows with discounted Akcijska MPC whose validity start date is after the report generation date.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Confirm these are valid customer-facing filter/spec values before exposing as filters.</t>
+          <t>Keep future sale prices inactive until the campaign starts.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>Suspicious placeholder values</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Detected values exactly matching placeholder tokens: 9, 0, /, -, N/A, NA.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Do not display these values publicly unless the client confirms the value is meaningful.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Numeric action-date values</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Rows where action validity date fields are plain numbers in the exported workbook.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>If present, ask whether Excel serial dates should be converted for display; keep source values unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Repeated non-descriptive review: Kolekcija (brend)</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>210019, 210003, 210022, 1040, 210000, 210001, 1033, 210009, 1034, 1095, 1035, 210013, 210011, 210012, 210010, 1112, 210020, 210024, 1075, 1044, 1074, 1076, 210006, 210023, 1045, 1106, 210014, 1049, 1053, 210025, 210016, 210015, 210017, 210018, 210021, 1037, 1036, 1097, 1096, 1109, 210002, 1080, 1078, 1077, 1039, 1079, 1110, 210004, 210005, 1098, 1041, 1099, 1100, 1101, 1042, 1043, 210007, 1038, 1050, 1115, 1048, 1047, 1046, 210008, 1011, 1014, 1010, 1013, 1009, 1141, 1012, 1005, 1008, 1004, 1007, 1003, 1139, 1006, 1017, 1018 ... (+30 more)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>2, 3, 4, 5, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 33, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 54, 55, 56, 57, 58, 59, 60, 61, 62, 69, 70, 73, 74, 75, 76, 77, 81, 82, 88, 89, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99, 100, 101, 102, 103 ... (+30 more)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Frequently repeated values found: EVONEK (26), RAF (28), BEAUTECH (10), ORBITA (20), POMPEA MIMI (11), SPARKLE (15)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Confirm these are valid customer-facing filter/spec values before exposing as filters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Repeated non-descriptive review: Boja 1</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>210019, 210003, 1025, 1114, 210000, 210001, 1034, 210011, 210012, 1112, 210020, 210024, 1076, 210006, 210023, 1045, 210014, 1049, 1053, 1111, 210025, 210016, 210017, 210018, 1037, 1036, 1109, 210002, 1080, 1078, 1027, 1110, 210004, 210005, 1041, 1042, 1107, 1022, 1032, 1030, 1043, 210007, 1023, 1024, 1038, 1050, 1028, 1046, 210008, 1020, 1019, 1021, 1108, 1026, 1011, 1014, 1010, 1013, 1009, 1141, 1012, 1005, 1008, 1004, 1007, 1003, 1139, 1006, 1017, 1018, 1142, 1015, 1016, 1140, 1135, 1132, 210031, 1156, 1153, 1089 ... (+32 more)</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>2, 3, 6, 7, 9, 10, 13, 17, 18, 20, 21, 22, 26, 27, 28, 29, 31, 32, 33, 34, 35, 36, 38, 39, 41, 42, 45, 46, 47, 48, 52, 54, 55, 56, 58, 62, 63, 64, 66, 68, 69, 70, 71, 72, 73, 74, 78, 81, 82, 83, 84, 85, 86, 87, 88, 89, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99, 100, 101, 102, 103, 104, 105, 106, 107, 124, 125, 129, 131, 132, 134 ... (+32 more)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Frequently repeated values found: crna (37), bela (29), siva (29), plava (17)</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Confirm these are valid customer-facing filter/spec values before exposing as filters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>Repeated non-descriptive review: Boja 2</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B31" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>1116, 1033, 1080, 1152, 1153, 1083, 1089, 210026, 210027, 210028, 1085, 1159, 210029, 210032, 210033, 210034, 1157, 1084, 1145, 1147, 1151, 1150</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>8, 11, 47, 119, 132, 133, 134, 139, 140, 141, 142, 147, 149, 150, 151, 152, 154, 164, 173, 200, 202, 210</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Frequently repeated values found: crna (22)</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Confirm these are valid customer-facing filter/spec values before exposing as filters.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F27"/>
+  <autoFilter ref="A1:F31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20554,12 +20658,16 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -20578,12 +20686,16 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -20602,12 +20714,16 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -20626,12 +20742,16 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -20650,12 +20770,16 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -20674,12 +20798,16 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -20698,12 +20826,16 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -20722,12 +20854,16 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -20746,12 +20882,16 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -20770,12 +20910,16 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -20794,12 +20938,16 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -20818,12 +20966,16 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -20842,12 +20994,16 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -20866,12 +21022,16 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -20890,12 +21050,16 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -20914,12 +21078,16 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -20938,12 +21106,16 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -20962,12 +21134,16 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -20986,12 +21162,16 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="F66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -21010,12 +21190,16 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F67" s="2" t="inlineStr"/>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -21034,12 +21218,16 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -21058,12 +21246,16 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -21082,12 +21274,16 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -21106,12 +21302,16 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -21130,12 +21330,16 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -21154,12 +21358,16 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -21178,12 +21386,16 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -21202,12 +21414,16 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -21226,12 +21442,16 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -21250,12 +21470,16 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -21274,12 +21498,16 @@
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -21298,12 +21526,16 @@
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -21322,12 +21554,16 @@
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -21346,12 +21582,16 @@
         </is>
       </c>
       <c r="D81" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -21370,12 +21610,16 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -21394,12 +21638,16 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="F83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -21418,12 +21666,16 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="F84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -21442,12 +21694,16 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="F85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -21466,12 +21722,16 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -21490,12 +21750,16 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -21514,12 +21778,16 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="F88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -21538,12 +21806,16 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -21562,12 +21834,16 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="F90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -21586,12 +21862,16 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -21610,12 +21890,16 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -21634,12 +21918,16 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="F93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -21658,12 +21946,16 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="F94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -21682,12 +21974,16 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="F95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -21706,12 +22002,16 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -21730,12 +22030,16 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -21754,12 +22058,16 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -21778,12 +22086,16 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E99" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -21802,12 +22114,16 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -21826,12 +22142,16 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F101" s="2" t="inlineStr"/>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -21850,12 +22170,16 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -21874,12 +22198,16 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F103" s="2" t="inlineStr"/>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -21898,12 +22226,16 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F104" s="2" t="inlineStr"/>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -21922,12 +22254,16 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F105" s="2" t="inlineStr"/>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -21946,12 +22282,16 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -21970,12 +22310,16 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -21994,12 +22338,16 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F108" s="2" t="inlineStr"/>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -22018,12 +22366,16 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F109" s="2" t="inlineStr"/>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -22042,12 +22394,16 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F110" s="2" t="inlineStr"/>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -22066,12 +22422,16 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -22090,12 +22450,16 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -22114,12 +22478,16 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F113" s="2" t="inlineStr"/>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -22138,12 +22506,16 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F114" s="2" t="inlineStr"/>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -22162,12 +22534,16 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="F115" s="2" t="inlineStr"/>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -22186,12 +22562,16 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F116" s="2" t="inlineStr"/>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>broken:lfs_pointer_description</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">

</xml_diff>